<commit_message>
flight performance and tsa throughput transformation
</commit_message>
<xml_diff>
--- a/doc/data_mapping.xlsx
+++ b/doc/data_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MSDA\D610 (capstone)\Airport Congestion Prediction System\Task 2\Airport Congestion Prediction System\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{024E43BC-56F6-49CB-AAAC-C0229347814A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{395DCACB-14DA-4913-AEE9-63255A2234B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{15CAE275-7B9E-4644-9142-08B22041D878}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="51870" windowHeight="21150" activeTab="1" xr2:uid="{15CAE275-7B9E-4644-9142-08B22041D878}"/>
   </bookViews>
   <sheets>
     <sheet name="airport" sheetId="3" r:id="rId1"/>
@@ -712,13 +712,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C88F96-8BDB-4A69-9F70-BFB7B724F58B}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>53</v>
       </c>
@@ -726,7 +726,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -734,7 +734,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>87</v>
       </c>
@@ -742,7 +742,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>89</v>
       </c>
@@ -750,7 +750,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>91</v>
       </c>
@@ -758,7 +758,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>93</v>
       </c>
@@ -766,7 +766,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>95</v>
       </c>
@@ -774,7 +774,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>97</v>
       </c>
@@ -782,7 +782,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>99</v>
       </c>
@@ -790,7 +790,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -798,7 +798,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>61</v>
       </c>
@@ -806,7 +806,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>101</v>
       </c>
@@ -814,7 +814,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>103</v>
       </c>
@@ -831,13 +831,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3F9604D-ED43-478C-B41E-34CF0FC1BCEB}">
   <dimension ref="A1:B31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>53</v>
       </c>
@@ -845,7 +845,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -853,7 +853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -861,7 +861,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -869,7 +869,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -877,7 +877,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>79</v>
       </c>
@@ -885,7 +885,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -893,7 +893,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
@@ -901,7 +901,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
@@ -909,7 +909,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>81</v>
       </c>
@@ -917,7 +917,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
@@ -925,7 +925,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -933,7 +933,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
@@ -941,7 +941,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>10</v>
       </c>
@@ -949,7 +949,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
@@ -957,7 +957,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -965,7 +965,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
@@ -973,7 +973,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
@@ -981,7 +981,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>15</v>
       </c>
@@ -989,7 +989,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -997,7 +997,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>17</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>18</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>19</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>21</v>
       </c>
@@ -1037,7 +1037,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>22</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>23</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>24</v>
       </c>
@@ -1061,7 +1061,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>25</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>26</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>27</v>
       </c>
@@ -1087,19 +1087,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF185162-98E5-409A-8720-92F9A2DEFAEE}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="26.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="26.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>53</v>
       </c>
@@ -1112,7 +1113,7 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>55</v>
       </c>
@@ -1125,7 +1126,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>57</v>
       </c>
@@ -1138,7 +1139,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>59</v>
       </c>
@@ -1151,7 +1152,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>61</v>
       </c>
@@ -1164,7 +1165,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>63</v>
       </c>
@@ -1177,7 +1178,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>65</v>
       </c>
@@ -1190,7 +1191,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>67</v>
       </c>
@@ -1203,7 +1204,7 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>69</v>
       </c>
@@ -1216,7 +1217,7 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>71</v>
       </c>
@@ -1229,7 +1230,7 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>73</v>
       </c>
@@ -1242,7 +1243,7 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>75</v>
       </c>
@@ -1255,7 +1256,7 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>77</v>
       </c>

</xml_diff>